<commit_message>
up to pri 5661e15
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$140</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$146</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="454">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -697,6 +697,18 @@
     <t xml:space="preserve">sends &lt;cmd&gt; (1byte in HEX) and optional &lt;value&gt; (0-65535) and &lt;param&gt; (0-255) to Orbiter</t>
   </si>
   <si>
+    <t xml:space="preserve">lebrew(&lt;msg&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sends &lt;msg&gt; to the BLE connected RoastSeeNEXT device</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sr900(&lt;target&gt;[,&lt;value&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sends &lt;target&gt; command like ‘heat’ and ‘fan’, with optional int &lt;value&gt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">shellyrelay(n,b)</t>
   </si>
   <si>
@@ -1069,6 +1081,30 @@
   </si>
   <si>
     <t xml:space="preserve">sets the PID lookahead in seconds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidPositiveTargetMin(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets the PID positive target range minium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidPositiveTargetMax(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets the PID positive target range maximum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidNegativeTargetMin(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets the PID negative target range minium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidNegativeTargetMax(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets the PID negative target range maximum</t>
   </si>
   <si>
     <t xml:space="preserve">replayLookahead(&lt;int&gt;)</t>
@@ -1362,12 +1398,6 @@
     <t xml:space="preserve">shows/hides the events of the background profile</t>
   </si>
   <si>
-    <t xml:space="preserve">upload2RoastHubs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upload current loaded profile to RoastHubs</t>
-  </si>
-  <si>
     <t xml:space="preserve">zoom(&lt;x&gt;[,&lt;y&gt;])</t>
   </si>
   <si>
@@ -1420,6 +1450,12 @@
   </si>
   <si>
     <t xml:space="preserve">toolbar forward action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dashboard([&lt;bool&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">show/hides dashboard; without argument visibility is toggled</t>
   </si>
   <si>
     <t xml:space="preserve">RC Command</t>
@@ -1611,7 +1647,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1630,6 +1666,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1652,37 +1692,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1756,7 +1796,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.73"/>
@@ -1853,7 +1893,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.27"/>
@@ -1969,7 +2009,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2258,8 +2298,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -2269,8 +2309,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C185"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C1048576"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.54"/>
@@ -2753,7 +2793,7 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
+      <c r="B61" s="3" t="s">
         <v>217</v>
       </c>
       <c r="C61" s="1" t="s">
@@ -2761,7 +2801,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
+      <c r="B62" s="3" t="s">
         <v>219</v>
       </c>
       <c r="C62" s="1" t="s">
@@ -2772,52 +2812,52 @@
       <c r="A63" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="C63" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B66" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="C66" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C66" s="1" t="s">
+    </row>
+    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="C67" s="1" t="s">
+    </row>
+    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="3" t="s">
         <v>234</v>
       </c>
@@ -2890,25 +2930,25 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="1" t="s">
+      <c r="B77" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C78" s="1" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3" t="s">
         <v>257</v>
       </c>
@@ -2926,77 +2966,77 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3" t="s">
-        <v>131</v>
+        <v>261</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>132</v>
+        <v>262</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="1" t="s">
-        <v>261</v>
-      </c>
       <c r="B82" s="3" t="s">
-        <v>127</v>
+        <v>263</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="B84" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>132</v>
+        <v>266</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3" t="s">
-        <v>263</v>
+        <v>135</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>264</v>
+        <v>136</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3" t="s">
-        <v>265</v>
+        <v>137</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>266</v>
+        <v>138</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3040,65 +3080,65 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="1" t="s">
+      <c r="B95" s="3" t="s">
         <v>277</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>218</v>
+        <v>278</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="1" t="s">
-        <v>278</v>
+      <c r="B96" s="3" t="s">
+        <v>279</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>220</v>
+        <v>280</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>280</v>
+        <v>222</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="B98" s="3" t="s">
         <v>282</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>283</v>
+        <v>224</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B99" s="3" t="s">
+    </row>
+    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B101" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C101" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B100" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3119,26 +3159,26 @@
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="3" t="s">
-        <v>131</v>
+        <v>293</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>132</v>
+        <v>294</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="3" t="s">
-        <v>295</v>
+        <v>131</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>296</v>
+        <v>132</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3305,7 +3345,7 @@
       <c r="B127" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="C127" s="1" t="s">
+      <c r="C127" s="5" t="s">
         <v>338</v>
       </c>
     </row>
@@ -3313,7 +3353,7 @@
       <c r="B128" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="C128" s="1" t="s">
+      <c r="C128" s="5" t="s">
         <v>340</v>
       </c>
     </row>
@@ -3321,7 +3361,7 @@
       <c r="B129" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="C129" s="1" t="s">
+      <c r="C129" s="5" t="s">
         <v>342</v>
       </c>
     </row>
@@ -3335,74 +3375,74 @@
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3" t="s">
-        <v>133</v>
+        <v>345</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3" t="s">
-        <v>137</v>
+        <v>349</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>138</v>
+        <v>350</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="3" t="s">
-        <v>354</v>
+        <v>133</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="3" t="s">
-        <v>358</v>
+        <v>137</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>359</v>
+        <v>138</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3598,57 +3638,57 @@
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="1" t="s">
+      <c r="B164" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="B164" s="3" t="s">
+      <c r="C164" s="1" t="s">
         <v>409</v>
-      </c>
-      <c r="C164" s="1" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C165" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C166" s="1" t="s">
         <v>413</v>
-      </c>
-      <c r="C166" s="1" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C167" s="1" t="s">
         <v>415</v>
-      </c>
-      <c r="C167" s="1" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C168" s="1" t="s">
         <v>417</v>
-      </c>
-      <c r="C168" s="1" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="C169" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="C169" s="1" t="s">
+    </row>
+    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="3" t="s">
         <v>421</v>
       </c>
@@ -3666,125 +3706,176 @@
     </row>
     <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="3" t="s">
-        <v>244</v>
+        <v>425</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="3" t="s">
-        <v>253</v>
+        <v>431</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="1" t="s">
-        <v>431</v>
-      </c>
       <c r="B176" s="3" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B177" s="3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B178" s="3" t="s">
-        <v>413</v>
+        <v>248</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="1" t="s">
-        <v>436</v>
-      </c>
       <c r="B179" s="3" t="s">
-        <v>129</v>
+        <v>438</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>130</v>
+        <v>439</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B180" s="3" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B181" s="3" t="s">
-        <v>131</v>
+        <v>257</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>132</v>
+        <v>442</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="1" t="s">
+        <v>443</v>
+      </c>
       <c r="B182" s="3" t="s">
-        <v>133</v>
+        <v>435</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>134</v>
+        <v>444</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B183" s="3" t="s">
-        <v>135</v>
+        <v>445</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B184" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="C184" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B185" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B186" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B187" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C187" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B188" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B189" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B190" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C184" s="1" t="s">
+      <c r="C190" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B185" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="C185" s="1" t="s">
-        <v>441</v>
-      </c>
-    </row>
+    <row r="191" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B191" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C158" r:id="rId1" display="ETB@x"/>
+    <hyperlink ref="C163" r:id="rId1" display="set xy cursor clamp mode (shortcut key z) to 0: off, 1: BT@x, 2: ET@x, 3: BTB@x, 4: ETB@x"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Revert "up to pri 5661e15"
This reverts commit f16daced0325fa1d51d55c0ae68d89feb3de9856.
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$146</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$140</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="442">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -697,18 +697,6 @@
     <t xml:space="preserve">sends &lt;cmd&gt; (1byte in HEX) and optional &lt;value&gt; (0-65535) and &lt;param&gt; (0-255) to Orbiter</t>
   </si>
   <si>
-    <t xml:space="preserve">lebrew(&lt;msg&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sends &lt;msg&gt; to the BLE connected RoastSeeNEXT device</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sr900(&lt;target&gt;[,&lt;value&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sends &lt;target&gt; command like ‘heat’ and ‘fan’, with optional int &lt;value&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">shellyrelay(n,b)</t>
   </si>
   <si>
@@ -1081,30 +1069,6 @@
   </si>
   <si>
     <t xml:space="preserve">sets the PID lookahead in seconds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pidPositiveTargetMin(&lt;n&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sets the PID positive target range minium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pidPositiveTargetMax(&lt;n&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sets the PID positive target range maximum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pidNegativeTargetMin(&lt;n&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sets the PID negative target range minium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pidNegativeTargetMax(&lt;n&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sets the PID negative target range maximum</t>
   </si>
   <si>
     <t xml:space="preserve">replayLookahead(&lt;int&gt;)</t>
@@ -1398,6 +1362,12 @@
     <t xml:space="preserve">shows/hides the events of the background profile</t>
   </si>
   <si>
+    <t xml:space="preserve">upload2RoastHubs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload current loaded profile to RoastHubs</t>
+  </si>
+  <si>
     <t xml:space="preserve">zoom(&lt;x&gt;[,&lt;y&gt;])</t>
   </si>
   <si>
@@ -1450,12 +1420,6 @@
   </si>
   <si>
     <t xml:space="preserve">toolbar forward action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dashboard([&lt;bool&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">show/hides dashboard; without argument visibility is toggled</t>
   </si>
   <si>
     <t xml:space="preserve">RC Command</t>
@@ -1647,7 +1611,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1666,10 +1630,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1692,37 +1652,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1796,7 +1756,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.73"/>
@@ -1893,7 +1853,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.27"/>
@@ -2009,7 +1969,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -2298,8 +2258,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -2309,8 +2269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1048576"/>
-  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C185"/>
+  <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.54"/>
@@ -2793,7 +2753,7 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="3" t="s">
+      <c r="A61" s="1" t="s">
         <v>217</v>
       </c>
       <c r="C61" s="1" t="s">
@@ -2801,7 +2761,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="3" t="s">
+      <c r="A62" s="1" t="s">
         <v>219</v>
       </c>
       <c r="C62" s="1" t="s">
@@ -2812,52 +2772,52 @@
       <c r="A63" s="1" t="s">
         <v>221</v>
       </c>
+      <c r="B63" s="4" t="s">
+        <v>222</v>
+      </c>
       <c r="C63" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>225</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C65" s="1" t="s">
         <v>227</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="s">
-        <v>231</v>
-      </c>
       <c r="B67" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="C67" s="1" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="s">
-        <v>233</v>
-      </c>
       <c r="B68" s="3" t="s">
         <v>234</v>
       </c>
@@ -2930,25 +2890,25 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
+        <v>252</v>
+      </c>
       <c r="B77" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="1" t="s">
-        <v>256</v>
-      </c>
       <c r="B79" s="3" t="s">
         <v>257</v>
       </c>
@@ -2966,77 +2926,77 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="B82" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>262</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C84" s="1" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3" t="s">
-        <v>135</v>
+        <v>263</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>136</v>
+        <v>264</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3" t="s">
-        <v>137</v>
+        <v>265</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>138</v>
+        <v>266</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3080,65 +3040,65 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B95" s="3" t="s">
+      <c r="A95" s="1" t="s">
         <v>277</v>
       </c>
       <c r="C95" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B96" s="3" t="s">
-        <v>279</v>
-      </c>
       <c r="C96" s="1" t="s">
-        <v>280</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>222</v>
+        <v>280</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B98" s="3" t="s">
         <v>282</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>224</v>
+        <v>283</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>284</v>
+        <v>130</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="1" t="s">
+      <c r="B100" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="C100" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="C100" s="1" t="s">
+    </row>
+    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B101" s="3" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="1" t="s">
+      <c r="C101" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3159,26 +3119,26 @@
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="3" t="s">
-        <v>293</v>
+        <v>131</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>294</v>
+        <v>132</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="3" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="3" t="s">
-        <v>131</v>
+        <v>295</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>132</v>
+        <v>296</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3345,7 +3305,7 @@
       <c r="B127" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="C127" s="5" t="s">
+      <c r="C127" s="1" t="s">
         <v>338</v>
       </c>
     </row>
@@ -3353,7 +3313,7 @@
       <c r="B128" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="C128" s="5" t="s">
+      <c r="C128" s="1" t="s">
         <v>340</v>
       </c>
     </row>
@@ -3361,7 +3321,7 @@
       <c r="B129" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="C129" s="5" t="s">
+      <c r="C129" s="1" t="s">
         <v>342</v>
       </c>
     </row>
@@ -3375,74 +3335,74 @@
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C131" s="1" t="s">
         <v>345</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>347</v>
-      </c>
-      <c r="C132" s="1" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3" t="s">
-        <v>349</v>
+        <v>137</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>350</v>
+        <v>138</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="3" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="3" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="3" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="3" t="s">
-        <v>133</v>
+        <v>354</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="3" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="3" t="s">
-        <v>137</v>
+        <v>358</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>138</v>
+        <v>359</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,57 +3598,57 @@
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1" t="s">
+        <v>408</v>
+      </c>
       <c r="B164" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="1" t="s">
-        <v>420</v>
-      </c>
       <c r="B170" s="3" t="s">
         <v>421</v>
       </c>
@@ -3706,176 +3666,125 @@
     </row>
     <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C172" s="1" t="s">
         <v>425</v>
-      </c>
-      <c r="C172" s="1" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="C173" s="1" t="s">
         <v>427</v>
-      </c>
-      <c r="C173" s="1" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="C174" s="1" t="s">
         <v>429</v>
-      </c>
-      <c r="C174" s="1" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="C175" s="1" t="s">
+      <c r="B176" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C176" s="1" t="s">
         <v>432</v>
-      </c>
-    </row>
-    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B176" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="C176" s="1" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B177" s="3" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B178" s="3" t="s">
-        <v>248</v>
+        <v>413</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="1" t="s">
+        <v>436</v>
+      </c>
       <c r="B179" s="3" t="s">
-        <v>438</v>
+        <v>129</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>439</v>
+        <v>130</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B180" s="3" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B181" s="3" t="s">
-        <v>257</v>
+        <v>131</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>442</v>
+        <v>132</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A182" s="1" t="s">
-        <v>443</v>
-      </c>
       <c r="B182" s="3" t="s">
-        <v>435</v>
+        <v>133</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>444</v>
+        <v>134</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B183" s="3" t="s">
-        <v>445</v>
+        <v>135</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B184" s="3" t="s">
-        <v>425</v>
+        <v>137</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>447</v>
+        <v>138</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A185" s="1" t="s">
-        <v>448</v>
-      </c>
       <c r="B185" s="3" t="s">
-        <v>129</v>
+        <v>440</v>
       </c>
       <c r="C185" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="186" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B186" s="3" t="s">
-        <v>449</v>
-      </c>
-      <c r="C186" s="1" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="187" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B187" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C187" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="188" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B188" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C188" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="189" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B189" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C189" s="1" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="190" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B190" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C190" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="191" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B191" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="C191" s="1" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>441</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C163" r:id="rId1" display="set xy cursor clamp mode (shortcut key z) to 0: off, 1: BT@x, 2: ET@x, 3: BTB@x, 4: ETB@x"/>
+    <hyperlink ref="C158" r:id="rId1" display="ETB@x"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>